<commit_message>
Add Pinnacle Communications contact, clean up hand-added rows
- Folded Trista Stillwagon (Pinnacle Communications) into the existing
  Pinnacle placeholder row with phone/email
- Normalized phone/address formatting on rows added since the last pass
  (Iceberg estimator, Rapid Hotel Supplies, RK Design Hospitality)
- Cleared the scratch-paste block now that it's in the table

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -2,22 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-255" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Contacts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,30 +27,38 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="16"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00595959"/>
+      <color rgb="FF595959"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00808080"/>
+      <color rgb="FF808080"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -63,12 +70,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
   </fills>
@@ -82,23 +89,25 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="FFBFBFBF"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -115,15 +124,29 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFF2CC"/>
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -201,8 +224,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J40" headerRowCount="1">
-  <autoFilter ref="A5:J40"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J43" headerRowCount="1">
+  <autoFilter ref="A5:J43"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Organization"/>
@@ -508,22 +531,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="21.85546875" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="36" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="20.25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>H2SEP — Contact List</t>
@@ -544,7 +567,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
+    <row r="5" ht="26.1" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Category</t>
@@ -602,105 +625,105 @@
           <t>Engineer</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Triun, LLC</t>
-        </is>
-      </c>
+      <c r="B6" s="5" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Edward R. De La Garza</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>(210) 572-4900</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>edelagarza@triunco.com</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
-        </is>
-      </c>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="6" t="inlineStr">
         <is>
-          <t>Carried from old list Engineer section, marked "UPDATED — Terminated by GC"</t>
+          <t>Open slot — add current engineer of record</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="n"/>
+          <t>Architect</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>MWT</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Anita Bansal</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>AIA, NCARB</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>(716) 435-0019</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>anita@mwtusa.com</t>
+        </is>
+      </c>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="7" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Open slot — add current engineer of record</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+      <c r="J7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="25.5" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Contractor (GC)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>MWT</t>
+          <t>Triun, LLC</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>General contractor</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Anita Bansal</t>
+          <t>Edward R. De La Garza</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>AIA, NCARB</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>(716) 435-0019</t>
+          <t>(210) 572-4900</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>anita@mwtusa.com</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n"/>
+          <t>edelagarza@triunco.com</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
+        </is>
+      </c>
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="6" t="n"/>
     </row>
-    <row r="9">
+    <row r="9" ht="25.5" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Contractor (GC)</t>
@@ -718,22 +741,22 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Edward R. De La Garza</t>
+          <t>Cesar Esquivel</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>General Superintendent</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>(210) 572-4900</t>
+          <t>(210) 718-1001</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>edelagarza@triunco.com</t>
+          <t>cesquivel@triunco.com</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
@@ -744,7 +767,7 @@
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="6" t="n"/>
     </row>
-    <row r="10">
+    <row r="10" ht="25.5" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Contractor (GC)</t>
@@ -762,22 +785,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Cesar Esquivel</t>
+          <t>Joaquin Gomez</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>General Superintendent</t>
+          <t>Superintendent</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>(210) 718-1001</t>
+          <t>(830) 335-0522</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>cesquivel@triunco.com</t>
+          <t>jgomez@triunco.com</t>
         </is>
       </c>
       <c r="H10" s="6" t="inlineStr">
@@ -788,7 +811,7 @@
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="6" t="n"/>
     </row>
-    <row r="11">
+    <row r="11" ht="25.5" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Contractor (GC)</t>
@@ -806,22 +829,22 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Joaquin Gomez</t>
+          <t>Morgan Davis</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Superintendent</t>
+          <t>Project Manager I</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>(830) 335-0522</t>
+          <t>(512) 771-2329</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>jgomez@triunco.com</t>
+          <t>mdavis@triunco.com</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
@@ -832,7 +855,7 @@
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Contractor (GC)</t>
@@ -850,73 +873,73 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Morgan Davis</t>
+          <t>Austin Jones</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Project Manager I</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>(512) 771-2329</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>mdavis@triunco.com</t>
-        </is>
-      </c>
+          <t>Project Manager / QC Coordinator</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="6" t="inlineStr">
         <is>
           <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
         </is>
       </c>
       <c r="I12" s="7" t="n"/>
-      <c r="J12" s="6" t="n"/>
-    </row>
-    <row r="13">
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>Added — fill in phone/email</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="25.5" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Triun, LLC</t>
+          <t>Iceberg Heating &amp; Air Conditioning</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>General contractor</t>
+          <t>Mechanical / HVAC</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Austin Jones</t>
+          <t>Jorge Garcia</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Project Manager / QC Coordinator</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="6" t="n"/>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>(817) 920-9950</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
+          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
         </is>
       </c>
       <c r="I13" s="7" t="n"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Added — fill in phone/email</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
+      <c r="J13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="25.5" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
           <t>MEP</t>
@@ -934,12 +957,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Jorge Garcia</t>
+          <t>Andrea Garcia</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Estimator</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -947,14 +970,14 @@
           <t>(817) 920-9950</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>estimating@icebergair.com</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
+          <t>1220 Oak Knoll Dr. Suite 200, Fort Worth, TX 76117</t>
         </is>
       </c>
       <c r="I14" s="7" t="n"/>
@@ -991,7 +1014,7 @@
           <t>(956) 309-4209</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G15" s="8" t="inlineStr">
         <is>
           <t>manuel@unitedelectricrgv.com</t>
         </is>
@@ -1048,7 +1071,7 @@
       <c r="I16" s="7" t="n"/>
       <c r="J16" s="6" t="n"/>
     </row>
-    <row r="17">
+    <row r="17" ht="25.5" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>MEP</t>
@@ -1140,7 +1163,7 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="6" t="n"/>
     </row>
-    <row r="19">
+    <row r="19" ht="25.5" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1224,7 +1247,7 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="6" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="25.5" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1268,7 +1291,7 @@
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="6" t="n"/>
     </row>
-    <row r="22">
+    <row r="22" ht="25.5" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1488,7 +1511,7 @@
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="6" t="n"/>
     </row>
-    <row r="27">
+    <row r="27" ht="25.5" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1620,7 +1643,7 @@
       <c r="I29" s="7" t="n"/>
       <c r="J29" s="6" t="n"/>
     </row>
-    <row r="30">
+    <row r="30" ht="25.5" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1664,7 +1687,7 @@
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="6" t="n"/>
     </row>
-    <row r="31">
+    <row r="31" ht="25.5" customHeight="1">
       <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1836,7 +1859,7 @@
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="6" t="n"/>
     </row>
-    <row r="35">
+    <row r="35" ht="25.5" customHeight="1">
       <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1862,9 +1885,10 @@
           <t>Project Coordinator</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>Direct: (847) 881-3681; Office: (847) 306-3777 Ext. 8603</t>
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>Direct: (847) 881-3681; 
+Office: (847) 306-3777 Ext. 8603</t>
         </is>
       </c>
       <c r="G35" s="6" t="n"/>
@@ -1924,7 +1948,7 @@
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="6" t="n"/>
     </row>
-    <row r="37">
+    <row r="37" ht="25.5" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1932,23 +1956,39 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Pinnacle</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="6" t="n"/>
+          <t>Pinnacle Communications</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Trista Stillwagon</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Project Coordinator</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>tstillwagon@pinn360.com</t>
+        </is>
+      </c>
       <c r="H37" s="6" t="n"/>
       <c r="I37" s="7" t="n"/>
-      <c r="J37" s="6" t="inlineStr">
-        <is>
-          <t>From notes at bottom of old list ("Pinnicle") — needs full contact info</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
+      <c r="J37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="25.5" customHeight="1">
       <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Subcontractor</t>
@@ -1980,33 +2020,37 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>National Wholesale Hospitality</t>
+          <t>Rapid Hotel Supplies</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>FF&amp;E</t>
+          <t>Appliances</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Royal West</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="n"/>
+          <t>Andy Kumar</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>(817) 723-5004</t>
-        </is>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>r.west@nws-inc.com</t>
+          <t>(213) 214-1739; Office: (866) 663-3301</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>sales01@rapidhotelsupplies.com</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+          <t>8910 Lawndale St. Suite C Houston, TX 77012</t>
         </is>
       </c>
       <c r="I39" s="7" t="n"/>
@@ -2020,64 +2064,211 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FF&amp;E </t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Ana Najera</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>(614) 933-0300 x1006</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>ana@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I40" s="7" t="n"/>
+      <c r="J40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="25.5" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FF&amp;E </t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Nadia Hayek</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Director of Design</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+        </is>
+      </c>
+      <c r="G41" s="9" t="inlineStr">
+        <is>
+          <t>nadia@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I41" s="7" t="n"/>
+      <c r="J41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="25.5" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>National Wholesale Hospitality</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Royal West</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n"/>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>(817) 723-5004</t>
+        </is>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>r.west@nws-inc.com</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+        </is>
+      </c>
+      <c r="I42" s="7" t="n"/>
+      <c r="J42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="25.5" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
           <t>Vingcard | ASSA ABLOY</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Door locks / access</t>
         </is>
       </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Leah Johnson</t>
         </is>
       </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Mobile: (469) 507-0672; Tech Support: (800) 225-8464</t>
-        </is>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="E43" s="5" t="n"/>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>Mobile: (469) 507-0672; 
+Tech Support: (800) 225-8464</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>leah.johnson@assaabloy.com</t>
         </is>
       </c>
-      <c r="H40" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
         </is>
       </c>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="6" t="inlineStr">
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — assaabloyglobalsolutions.com</t>
         </is>
       </c>
     </row>
+    <row r="44"/>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
   </sheetData>
-  <conditionalFormatting sqref="C6:H40">
-    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+  <conditionalFormatting sqref="B6:H43">
+    <cfRule type="expression" priority="2" dxfId="0">
+      <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:H43">
+    <cfRule type="expression" priority="1" dxfId="0">
       <formula>AND(ISBLANK(C6),$B6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B6:H40">
-    <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
-      <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="A6:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick a category from the list." type="list">
+    <dataValidation sqref="A6:A203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick a category from the list." type="list">
       <formula1>"Owner,Engineer,Architect,Contractor (GC),MEP,Structural,Subcontractor,Supplier,Consultant,Inspector / AHJ"</formula1>
     </dataValidation>
-    <dataValidation sqref="I6:I200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I6:I203" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N/A"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId5"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add APM Services LLC contacts (Ramón Aguirre, Jacob Murphy)
Inserted into the Subcontractor section; scope/trade left blank pending
confirmation. No email on file yet for Ramón Aguirre.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -79,7 +79,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -102,12 +102,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,12 +144,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -147,6 +170,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF2CC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -224,8 +254,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J43" headerRowCount="1">
-  <autoFilter ref="A5:J43"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J45" headerRowCount="1">
+  <autoFilter ref="A5:J45"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Organization"/>
@@ -531,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -567,6 +597,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="26.1" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -2013,92 +2044,68 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>Rapid Hotel Supplies</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr">
-        <is>
-          <t>Appliances</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>Andy Kumar</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Sales Manager</t>
-        </is>
-      </c>
-      <c r="F39" s="5" t="inlineStr">
-        <is>
-          <t>(213) 214-1739; Office: (866) 663-3301</t>
-        </is>
-      </c>
-      <c r="G39" s="9" t="inlineStr">
-        <is>
-          <t>sales01@rapidhotelsupplies.com</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
-        <is>
-          <t>8910 Lawndale St. Suite C Houston, TX 77012</t>
-        </is>
-      </c>
-      <c r="I39" s="7" t="n"/>
-      <c r="J39" s="6" t="n"/>
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>APM Services LLC</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>Ramón Aguirre</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="F39" s="10" t="inlineStr">
+        <is>
+          <t>(305) 988-2350; (512) 887-7980</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="11" t="n"/>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="11" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>RK Design Hospitality</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FF&amp;E </t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>Ana Najera</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>(614) 933-0300 x1006</t>
-        </is>
-      </c>
-      <c r="G40" s="9" t="inlineStr">
-        <is>
-          <t>ana@rkhdesign.com</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
-        </is>
-      </c>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="6" t="n"/>
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>APM Services LLC</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>Jacob Murphy</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="n"/>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>(830) 752-2023</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>murphyisme@live.com</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="n"/>
+      <c r="I40" s="12" t="n"/>
+      <c r="J40" s="11" t="n"/>
     </row>
     <row r="41" ht="25.5" customHeight="1">
       <c r="A41" s="5" t="inlineStr">
@@ -2108,37 +2115,37 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
+          <t>Rapid Hotel Supplies</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FF&amp;E </t>
+          <t>Appliances</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Nadia Hayek</t>
+          <t>Andy Kumar</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Director of Design</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+          <t>(213) 214-1739; Office: (866) 663-3301</t>
         </is>
       </c>
       <c r="G41" s="9" t="inlineStr">
         <is>
-          <t>nadia@rkhdesign.com</t>
+          <t>sales01@rapidhotelsupplies.com</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>8910 Lawndale St. Suite C Houston, TX 77012</t>
         </is>
       </c>
       <c r="I41" s="7" t="n"/>
@@ -2152,33 +2159,37 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>National Wholesale Hospitality</t>
+          <t>RK Design Hospitality</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>FF&amp;E</t>
+          <t xml:space="preserve">FF&amp;E </t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Royal West</t>
-        </is>
-      </c>
-      <c r="E42" s="5" t="n"/>
+          <t>Ana Najera</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>(817) 723-5004</t>
-        </is>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
-        <is>
-          <t>r.west@nws-inc.com</t>
+          <t>(614) 933-0300 x1006</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>ana@rkhdesign.com</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I42" s="7" t="n"/>
@@ -2192,62 +2203,135 @@
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FF&amp;E </t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Nadia Hayek</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Director of Design</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+        </is>
+      </c>
+      <c r="G43" s="9" t="inlineStr">
+        <is>
+          <t>nadia@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I43" s="7" t="n"/>
+      <c r="J43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>National Wholesale Hospitality</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Royal West</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>(817) 723-5004</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>r.west@nws-inc.com</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+        </is>
+      </c>
+      <c r="I44" s="7" t="n"/>
+      <c r="J44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
           <t>Vingcard | ASSA ABLOY</t>
         </is>
       </c>
-      <c r="C43" s="6" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>Door locks / access</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Leah Johnson</t>
         </is>
       </c>
-      <c r="E43" s="5" t="n"/>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="6" t="inlineStr">
         <is>
           <t>Mobile: (469) 507-0672; 
 Tech Support: (800) 225-8464</t>
         </is>
       </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>leah.johnson@assaabloy.com</t>
         </is>
       </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
         </is>
       </c>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="6" t="inlineStr">
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — assaabloyglobalsolutions.com</t>
         </is>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
   </sheetData>
-  <conditionalFormatting sqref="B6:H43">
-    <cfRule type="expression" priority="2" dxfId="0">
+  <conditionalFormatting sqref="B6:H45">
+    <cfRule type="expression" priority="1" dxfId="2" stopIfTrue="0">
       <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:H43">
-    <cfRule type="expression" priority="1" dxfId="0">
+  <conditionalFormatting sqref="C6:H45">
+    <cfRule type="expression" priority="2" dxfId="2" stopIfTrue="0">
       <formula>AND(ISBLANK(C6),$B6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2262,9 +2346,9 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G39" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G40" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Add Annalisa Call (Texas Chutes LLC administrative assistant)
Inserted next to the existing Texas Chutes / Gerry Whitaker row.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -121,7 +121,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,6 +149,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -254,8 +260,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J45" headerRowCount="1">
-  <autoFilter ref="A5:J45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J46" headerRowCount="1">
+  <autoFilter ref="A5:J46"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Organization"/>
@@ -561,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1719,48 +1725,48 @@
       <c r="J30" s="6" t="n"/>
     </row>
     <row r="31" ht="25.5" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t>Subcontractor</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Keepers Construction</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Flooring</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Justin Allen Perez</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>(210) 909-3250</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>keeperconst@gmail.com</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
-        </is>
-      </c>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="6" t="n"/>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>Texas Chutes</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Trash / linen chutes</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Annalisa Call</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Administrative Assistant</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>(830) 964-3102</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>14812 S. Access Road, Unit A, Canyon Lake, TX 78133</t>
+        </is>
+      </c>
+      <c r="I31" s="14" t="n"/>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>www.texaschutes.com</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1770,17 +1776,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Velasquez Pool</t>
+          <t>Keepers Construction</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Pool</t>
+          <t>Flooring</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Sabino Velasquez</t>
+          <t>Justin Allen Perez</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1790,17 +1796,17 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>(830) 352-4026</t>
+          <t>(210) 909-3250</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>velasquezpools@yahoo.com</t>
+          <t>keeperconst@gmail.com</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
+          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I32" s="7" t="n"/>
@@ -1814,17 +1820,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Cemplex Group</t>
+          <t>Velasquez Pool</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Gypsum floor underlayment</t>
+          <t>Pool</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Shane Kuempel</t>
+          <t>Sabino Velasquez</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1834,17 +1840,17 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>(817) 760-9457</t>
+          <t>(830) 352-4026</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>skuempel@cemplexgroup.com</t>
+          <t>velasquezpools@yahoo.com</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
+          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I33" s="7" t="n"/>
@@ -1858,33 +1864,37 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Access Online Inc</t>
+          <t>Cemplex Group</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Data / low voltage</t>
+          <t>Gypsum floor underlayment</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Rameez</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="n"/>
+          <t>Shane Kuempel</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>(847) 306-3777 Ext. 8205</t>
+          <t>(817) 760-9457</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>rameez@accessonline.io</t>
+          <t>skuempel@cemplexgroup.com</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>2130 Foster Ave., Wheeling, IL 60090</t>
+          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
         </is>
       </c>
       <c r="I34" s="7" t="n"/>
@@ -1908,76 +1918,72 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
+          <t>Rameez</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>(847) 306-3777 Ext. 8205</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>rameez@accessonline.io</t>
+        </is>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
+        <is>
+          <t>2130 Foster Ave., Wheeling, IL 60090</t>
+        </is>
+      </c>
+      <c r="I35" s="7" t="n"/>
+      <c r="J35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>Access Online Inc</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Data / low voltage</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
           <t>Bhavana Rao</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>Project Coordinator</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>Direct: (847) 881-3681; 
 Office: (847) 306-3777 Ext. 8603</t>
         </is>
       </c>
-      <c r="G35" s="6" t="n"/>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>2130 Foster Ave., Wheeling, IL 60090</t>
         </is>
       </c>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="6" t="inlineStr">
+      <c r="I36" s="7" t="n"/>
+      <c r="J36" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — get email</t>
         </is>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
-        <is>
-          <t>Subcontractor</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>The Green Company</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Landscaping</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Jorge Cavazos</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>(830) 335-2488</t>
-        </is>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>management@thegreencoep.com</t>
-        </is>
-      </c>
-      <c r="H36" s="6" t="inlineStr">
-        <is>
-          <t>126 Concho Street, Eagle Pass, TX 78852</t>
-        </is>
-      </c>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="6" t="n"/>
     </row>
     <row r="37" ht="25.5" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
@@ -1987,35 +1993,39 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Pinnacle Communications</t>
+          <t>The Green Company</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Landscaping</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Trista Stillwagon</t>
+          <t>Jorge Cavazos</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Project Coordinator</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
+          <t>(830) 335-2488</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>tstillwagon@pinn360.com</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="n"/>
+          <t>management@thegreencoep.com</t>
+        </is>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
+        <is>
+          <t>126 Concho Street, Eagle Pass, TX 78852</t>
+        </is>
+      </c>
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="6" t="n"/>
     </row>
@@ -2027,53 +2037,61 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>AMI</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="n"/>
-      <c r="D38" s="5" t="n"/>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="6" t="n"/>
+          <t>Pinnacle Communications</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Communications</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Trista Stillwagon</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Project Coordinator</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>tstillwagon@pinn360.com</t>
+        </is>
+      </c>
       <c r="H38" s="6" t="n"/>
       <c r="I38" s="7" t="n"/>
-      <c r="J38" s="6" t="inlineStr">
+      <c r="J38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>AMI</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="7" t="n"/>
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — needs full contact info</t>
         </is>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Subcontractor</t>
-        </is>
-      </c>
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>APM Services LLC</t>
-        </is>
-      </c>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="10" t="inlineStr">
-        <is>
-          <t>Ramón Aguirre</t>
-        </is>
-      </c>
-      <c r="E39" s="10" t="inlineStr">
-        <is>
-          <t>President</t>
-        </is>
-      </c>
-      <c r="F39" s="10" t="inlineStr">
-        <is>
-          <t>(305) 988-2350; (512) 887-7980</t>
-        </is>
-      </c>
-      <c r="G39" s="11" t="n"/>
-      <c r="H39" s="11" t="n"/>
-      <c r="I39" s="12" t="n"/>
-      <c r="J39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -2089,67 +2107,55 @@
       <c r="C40" s="11" t="n"/>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Jacob Murphy</t>
-        </is>
-      </c>
-      <c r="E40" s="10" t="n"/>
+          <t>Ramón Aguirre</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>(830) 752-2023</t>
-        </is>
-      </c>
-      <c r="G40" s="11" t="inlineStr">
-        <is>
-          <t>murphyisme@live.com</t>
-        </is>
-      </c>
+          <t>(305) 988-2350; (512) 887-7980</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="n"/>
       <c r="H40" s="11" t="n"/>
       <c r="I40" s="12" t="n"/>
       <c r="J40" s="11" t="n"/>
     </row>
     <row r="41" ht="25.5" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>Rapid Hotel Supplies</t>
-        </is>
-      </c>
-      <c r="C41" s="6" t="inlineStr">
-        <is>
-          <t>Appliances</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>Andy Kumar</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Sales Manager</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>(213) 214-1739; Office: (866) 663-3301</t>
-        </is>
-      </c>
-      <c r="G41" s="9" t="inlineStr">
-        <is>
-          <t>sales01@rapidhotelsupplies.com</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
-        <is>
-          <t>8910 Lawndale St. Suite C Houston, TX 77012</t>
-        </is>
-      </c>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="6" t="n"/>
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>Subcontractor</t>
+        </is>
+      </c>
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>APM Services LLC</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>Jacob Murphy</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="inlineStr">
+        <is>
+          <t>(830) 752-2023</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>murphyisme@live.com</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="n"/>
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="11" t="n"/>
     </row>
     <row r="42" ht="25.5" customHeight="1">
       <c r="A42" s="5" t="inlineStr">
@@ -2159,37 +2165,37 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
+          <t>Rapid Hotel Supplies</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">FF&amp;E </t>
+          <t>Appliances</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Ana Najera</t>
+          <t>Andy Kumar</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>(614) 933-0300 x1006</t>
+          <t>(213) 214-1739; Office: (866) 663-3301</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>ana@rkhdesign.com</t>
+          <t>sales01@rapidhotelsupplies.com</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>8910 Lawndale St. Suite C Houston, TX 77012</t>
         </is>
       </c>
       <c r="I42" s="7" t="n"/>
@@ -2213,22 +2219,22 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Nadia Hayek</t>
+          <t>Ana Najera</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Director of Design</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+          <t>(614) 933-0300 x1006</t>
         </is>
       </c>
       <c r="G43" s="9" t="inlineStr">
         <is>
-          <t>nadia@rkhdesign.com</t>
+          <t>ana@rkhdesign.com</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
@@ -2247,33 +2253,37 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>National Wholesale Hospitality</t>
+          <t>RK Design Hospitality</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>FF&amp;E</t>
+          <t xml:space="preserve">FF&amp;E </t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Royal West</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="n"/>
+          <t>Nadia Hayek</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Director of Design</t>
+        </is>
+      </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>(817) 723-5004</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>r.west@nws-inc.com</t>
+          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+        </is>
+      </c>
+      <c r="G44" s="9" t="inlineStr">
+        <is>
+          <t>nadia@rkhdesign.com</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I44" s="7" t="n"/>
@@ -2287,50 +2297,90 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
+          <t>National Wholesale Hospitality</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Royal West</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="n"/>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>(817) 723-5004</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>r.west@nws-inc.com</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+        </is>
+      </c>
+      <c r="I45" s="7" t="n"/>
+      <c r="J45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
           <t>Vingcard | ASSA ABLOY</t>
         </is>
       </c>
-      <c r="C45" s="6" t="inlineStr">
+      <c r="C46" s="6" t="inlineStr">
         <is>
           <t>Door locks / access</t>
         </is>
       </c>
-      <c r="D45" s="5" t="inlineStr">
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Leah Johnson</t>
         </is>
       </c>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="E46" s="5" t="n"/>
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>Mobile: (469) 507-0672; 
 Tech Support: (800) 225-8464</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>leah.johnson@assaabloy.com</t>
         </is>
       </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
         </is>
       </c>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="6" t="inlineStr">
+      <c r="I46" s="7" t="n"/>
+      <c r="J46" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — assaabloyglobalsolutions.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:H45">
+  <conditionalFormatting sqref="B6:H46">
     <cfRule type="expression" priority="1" dxfId="2" stopIfTrue="0">
       <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:H45">
+  <conditionalFormatting sqref="C6:H46">
     <cfRule type="expression" priority="2" dxfId="2" stopIfTrue="0">
       <formula>AND(ISBLANK(C6),$B6&lt;&gt;"")</formula>
     </cfRule>
@@ -2346,9 +2396,9 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G41" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G42" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G43" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G44" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Sync contact list with latest live edits from Google Sheets
Austin Jones' title updated to Assistant Project Manager, and the
Andres Garza placeholder row removed — both edited directly in the
Google Sheets copy since the last sync.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -201,8 +201,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J54" headerRowCount="1">
-  <autoFilter ref="A5:J54"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J53" headerRowCount="1">
+  <autoFilter ref="A5:J53"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Organization"/>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -855,7 +855,7 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Project Manager / QC Coordinator</t>
+          <t>Assistant Project Manager</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -879,38 +879,46 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Triun, LLC</t>
+          <t>Iceberg Heating &amp; Air Conditioning</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>General contractor</t>
+          <t>Mechanical / HVAC</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Andres Garza</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="6" t="n"/>
+          <t>Jorge Garcia</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>(817) 920-9950</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
+        </is>
+      </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
+          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
         </is>
       </c>
       <c r="I13" s="7" t="n"/>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Fill in title, phone, email</t>
-        </is>
-      </c>
+      <c r="J13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -930,12 +938,12 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Jorge Garcia</t>
+          <t>Andrea Garcia</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Estimator</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -945,12 +953,12 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
+          <t>estimating@icebergair.com</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
+          <t>1220 Oak Knoll Dr. Suite 200, Fort Worth, TX 76117</t>
         </is>
       </c>
       <c r="I14" s="7" t="n"/>
@@ -964,37 +972,37 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Iceberg Heating &amp; Air Conditioning</t>
+          <t>United Electric</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Mechanical / HVAC</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Andrea Garcia</t>
+          <t>Manuel Hernandez</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Estimator</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>(817) 920-9950</t>
+          <t>(956) 309-4209</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>estimating@icebergair.com</t>
+          <t>manuel@unitedelectricrgv.com</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>1220 Oak Knoll Dr. Suite 200, Fort Worth, TX 76117</t>
+          <t>4624 Martinal Road, Brownsville, TX 78526</t>
         </is>
       </c>
       <c r="I15" s="7" t="n"/>
@@ -1008,17 +1016,17 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>United Electric</t>
+          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Manuel Hernandez</t>
+          <t>Larry Sanchez</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1028,17 +1036,17 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>(956) 309-4209</t>
+          <t>(830) 513-1789</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>manuel@unitedelectricrgv.com</t>
+          <t>larrysplumbing@live.com</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>4624 Martinal Road, Brownsville, TX 78526</t>
+          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I16" s="7" t="n"/>
@@ -1062,12 +1070,12 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Larry Sanchez</t>
+          <t>Jay Hernandaz</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Foreman</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
@@ -1086,95 +1094,95 @@
         </is>
       </c>
       <c r="I17" s="7" t="n"/>
-      <c r="J17" s="6" t="n"/>
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>From notes at bottom of old list — verify name spelling and get direct number</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
+          <t>Steel Tech USA</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Steel erection</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Jay Hernandaz</t>
+          <t>Yalcin Kucukkomurler</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Foreman</t>
+          <t>Director of Engineering</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>(830) 513-1789</t>
+          <t>(561) 906-2840</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>larrysplumbing@live.com</t>
+          <t>yalcin@steeltechusa.com</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
+          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
         </is>
       </c>
       <c r="I18" s="7" t="n"/>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>From notes at bottom of old list — verify name spelling and get direct number</t>
-        </is>
-      </c>
+      <c r="J18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>Subcontractor</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Steel Tech USA</t>
+          <t>A/E Hiller &amp; Sons Inc.</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Steel erection</t>
+          <t>Concrete; parking lot striping &amp; signage; ADA pavers</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Yalcin Kucukkomurler</t>
+          <t>Christopher Hiller</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Director of Engineering</t>
+          <t>President</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>(561) 906-2840</t>
+          <t>(830) 773-9156</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>yalcin@steeltechusa.com</t>
+          <t>cw_hiller@yahoo.com</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
+          <t>P.O. Box 557, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I19" s="7" t="n"/>
@@ -1188,37 +1196,33 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>A/E Hiller &amp; Sons Inc.</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Concrete; parking lot striping &amp; signage; ADA pavers</t>
-        </is>
-      </c>
+          <t>JC Enterprises</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="n"/>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Christopher Hiller</t>
+          <t>Isaac Chapa</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>(830) 773-9156</t>
+          <t>(830) 968-1857</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>cw_hiller@yahoo.com</t>
+          <t>jcenterprises@yahoo.com</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>P.O. Box 557, Eagle Pass, TX 78852</t>
+          <t>2254 Foothills St., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I20" s="7" t="n"/>
@@ -1232,13 +1236,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>JC Enterprises</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="n"/>
+          <t>Texas Fire Services, LLC</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Fire protection</t>
+        </is>
+      </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Isaac Chapa</t>
+          <t>Rodney Jackson</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1248,17 +1256,17 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>(830) 968-1857</t>
+          <t>(830) 609-9090</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>jcenterprises@yahoo.com</t>
+          <t>rod@texasfireservices.net</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>2254 Foothills St., Eagle Pass, TX 78852</t>
+          <t>1260 FM 1863, Building 2, New Braunfels, TX 78132</t>
         </is>
       </c>
       <c r="I21" s="7" t="n"/>
@@ -1272,17 +1280,17 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Texas Fire Services, LLC</t>
+          <t>TK Elevator Corporation</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Fire protection</t>
+          <t>Elevator</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Rodney Jackson</t>
+          <t>WH (Joey) Hawkins Jr.</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1292,17 +1300,17 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>(830) 609-9090</t>
+          <t>(210) 669-4818</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>rod@texasfireservices.net</t>
+          <t>joey.hawkins@tkelevator.com</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>1260 FM 1863, Building 2, New Braunfels, TX 78132</t>
+          <t>3660 Thousand Oaks, Suite 210, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I22" s="7" t="n"/>
@@ -1316,17 +1324,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>TK Elevator Corporation</t>
+          <t>Irontek Metal Works</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Elevator</t>
+          <t>Misc. metals</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>WH (Joey) Hawkins Jr.</t>
+          <t>Johnny Pina</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1336,17 +1344,17 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>(210) 669-4818</t>
+          <t>(512) 633-5140</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>joey.hawkins@tkelevator.com</t>
+          <t>irontekmetalworks@gmail.com</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>3660 Thousand Oaks, Suite 210, San Antonio, TX 78247</t>
+          <t>213 Goldenrod, San Marcos, TX 78666</t>
         </is>
       </c>
       <c r="I23" s="7" t="n"/>
@@ -1360,17 +1368,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Irontek Metal Works</t>
+          <t>The Montecito</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Misc. metals</t>
+          <t>Stucco / plastering</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Johnny Pina</t>
+          <t>Victor A. Rodriguez</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1380,17 +1388,17 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>(512) 633-5140</t>
+          <t>(940) 600-8106</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>irontekmetalworks@gmail.com</t>
+          <t>plasteringstuccoirdallas@gmail.com</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>213 Goldenrod, San Marcos, TX 78666</t>
+          <t>5517 Rio Rd., Denton, TX 76208</t>
         </is>
       </c>
       <c r="I24" s="7" t="n"/>
@@ -1404,17 +1412,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>The Montecito</t>
+          <t>Keen Glass Solutions</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Stucco / plastering</t>
+          <t>Glass &amp; glazing</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Victor A. Rodriguez</t>
+          <t>Joe Wilkinson</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1424,17 +1432,17 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>(940) 600-8106</t>
+          <t>(214) 673-1761</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>plasteringstuccoirdallas@gmail.com</t>
+          <t>sales@keen-glass.org</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>5517 Rio Rd., Denton, TX 76208</t>
+          <t>3923 Morse St. #116, Denton, TX 76208</t>
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
@@ -1448,17 +1456,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Keen Glass Solutions</t>
+          <t>Thermal Guard Roofing</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Glass &amp; glazing</t>
+          <t>TPO roofing</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Joe Wilkinson</t>
+          <t>Quinton Rockwell</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1468,17 +1476,17 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>(214) 673-1761</t>
+          <t>(817) 909-9884</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>sales@keen-glass.org</t>
+          <t>quinton@thermalguardroofing.com</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>3923 Morse St. #116, Denton, TX 76208</t>
+          <t>P.O. Box 1026, Argyle, TX 76226</t>
         </is>
       </c>
       <c r="I26" s="7" t="n"/>
@@ -1492,17 +1500,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Thermal Guard Roofing</t>
+          <t>Security Integrated</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>TPO roofing</t>
+          <t>Security systems</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Quinton Rockwell</t>
+          <t>Randy Jasik</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1512,17 +1520,17 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>(817) 909-9884</t>
+          <t>(210) 519-5009</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>quinton@thermalguardroofing.com</t>
+          <t>team@siinc.systems</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>P.O. Box 1026, Argyle, TX 76226</t>
+          <t>14080 Nacogdoches Rd. #536, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I27" s="7" t="n"/>
@@ -1536,17 +1544,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Security Integrated</t>
+          <t>Tormax USA, LLC</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Security systems</t>
+          <t>Automatic glass doors</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Randy Jasik</t>
+          <t>Chris Valadez</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1556,17 +1564,17 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>(210) 519-5009</t>
+          <t>(210) 362-4887</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>team@siinc.systems</t>
+          <t>cvaladez@tormaxusa.com</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>14080 Nacogdoches Rd. #536, San Antonio, TX 78247</t>
+          <t>12859 Wetmore Road, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I28" s="7" t="n"/>
@@ -1580,17 +1588,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Tormax USA, LLC</t>
+          <t>Steel Tech USA</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Automatic glass doors</t>
+          <t>Steel fabrication</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Chris Valadez</t>
+          <t>Edward Tekin</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1600,17 +1608,17 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>(210) 362-4887</t>
+          <t>(254) 368-7956</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>cvaladez@tormaxusa.com</t>
+          <t>edward@steeltechusa.com</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>12859 Wetmore Road, San Antonio, TX 78247</t>
+          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
         </is>
       </c>
       <c r="I29" s="7" t="n"/>
@@ -1624,17 +1632,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Steel Tech USA</t>
+          <t>Texas Chutes</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Steel fabrication</t>
+          <t>Trash / linen chutes</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Edward Tekin</t>
+          <t>Gerry Whitaker</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1644,17 +1652,17 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>(254) 368-7956</t>
+          <t>(830) 964-3102</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>edward@steeltechusa.com</t>
+          <t>gerry@texaschutes.com</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
+          <t>14812 South Access Rd. #A, Canyon Lake, TX 78133</t>
         </is>
       </c>
       <c r="I30" s="7" t="n"/>
@@ -1678,12 +1686,12 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Gerry Whitaker</t>
+          <t>Annalisa Call</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Administrative Assistant</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1691,18 +1699,18 @@
           <t>(830) 964-3102</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>gerry@texaschutes.com</t>
-        </is>
-      </c>
+      <c r="G31" s="6" t="n"/>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>14812 South Access Rd. #A, Canyon Lake, TX 78133</t>
+          <t>14812 S. Access Road, Unit A, Canyon Lake, TX 78133</t>
         </is>
       </c>
       <c r="I31" s="7" t="n"/>
-      <c r="J31" s="6" t="n"/>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>www.texaschutes.com</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1712,41 +1720,41 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Texas Chutes</t>
+          <t>Keepers Construction</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Trash / linen chutes</t>
+          <t>Flooring</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Annalisa Call</t>
+          <t>Justin Allen Perez</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Administrative Assistant</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>(830) 964-3102</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="n"/>
+          <t>(210) 909-3250</t>
+        </is>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>keeperconst@gmail.com</t>
+        </is>
+      </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>14812 S. Access Road, Unit A, Canyon Lake, TX 78133</t>
+          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I32" s="7" t="n"/>
-      <c r="J32" s="6" t="inlineStr">
-        <is>
-          <t>www.texaschutes.com</t>
-        </is>
-      </c>
+      <c r="J32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -1756,17 +1764,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Keepers Construction</t>
+          <t>Velasquez Pool</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Flooring</t>
+          <t>Pool</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Justin Allen Perez</t>
+          <t>Sabino Velasquez</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1776,17 +1784,17 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>(210) 909-3250</t>
+          <t>(830) 352-4026</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>keeperconst@gmail.com</t>
+          <t>velasquezpools@yahoo.com</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
+          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I33" s="7" t="n"/>
@@ -1800,17 +1808,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Velasquez Pool</t>
+          <t>Cemplex Group</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Pool</t>
+          <t>Gypsum floor underlayment</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Sabino Velasquez</t>
+          <t>Shane Kuempel</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1820,17 +1828,17 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>(830) 352-4026</t>
+          <t>(817) 760-9457</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>velasquezpools@yahoo.com</t>
+          <t>skuempel@cemplexgroup.com</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
+          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
         </is>
       </c>
       <c r="I34" s="7" t="n"/>
@@ -1844,37 +1852,33 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Cemplex Group</t>
+          <t>Access Online Inc</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Gypsum floor underlayment</t>
+          <t>Data / low voltage</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Shane Kuempel</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Owner</t>
-        </is>
-      </c>
+          <t>Rameez</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>(817) 760-9457</t>
+          <t>(847) 306-3777 Ext. 8205</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>skuempel@cemplexgroup.com</t>
+          <t>rameez@accessonline.io</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
+          <t>2130 Foster Ave., Wheeling, IL 60090</t>
         </is>
       </c>
       <c r="I35" s="7" t="n"/>
@@ -1898,18 +1902,22 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Rameez</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="n"/>
+          <t>Bhavana Rao</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Project Coordinator</t>
+        </is>
+      </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>(847) 306-3777 Ext. 8205</t>
+          <t>Direct: (847) 881-3681; Office: (847) 306-3777 Ext. 8603</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>rameez@accessonline.io</t>
+          <t>bhavana.rao@accessonline.io</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
@@ -1928,37 +1936,37 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Access Online Inc</t>
+          <t>The Green Company</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Data / low voltage</t>
+          <t>Landscaping</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Bhavana Rao</t>
+          <t>Jorge Cavazos</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Project Coordinator</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>Direct: (847) 881-3681; Office: (847) 306-3777 Ext. 8603</t>
+          <t>(830) 335-2488</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>bhavana.rao@accessonline.io</t>
+          <t>management@thegreencoep.com</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>2130 Foster Ave., Wheeling, IL 60090</t>
+          <t>126 Concho Street, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I37" s="7" t="n"/>
@@ -1972,39 +1980,35 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>The Green Company</t>
+          <t>Pinnacle Communications</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Landscaping</t>
+          <t>Communications</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Jorge Cavazos</t>
+          <t>Trista Stillwagon</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Project Coordinator</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>(830) 335-2488</t>
+          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>management@thegreencoep.com</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr">
-        <is>
-          <t>126 Concho Street, Eagle Pass, TX 78852</t>
-        </is>
-      </c>
+          <t>tstillwagon@pinn360.com</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="n"/>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="6" t="n"/>
     </row>
@@ -2016,35 +2020,39 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Pinnacle Communications</t>
+          <t>Spectrum Business</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Internet / Fiber</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Trista Stillwagon</t>
+          <t>Ian V Rywalt</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Project Coordinator</t>
+          <t>Program Manager</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
+          <t>O: (407) 215-5917; M: (689) 213-9770</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>tstillwagon@pinn360.com</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="n"/>
+          <t>Ian.Rywalt@spectrum.com</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>65 S Keller Rd, Orlando, FL 32810</t>
+        </is>
+      </c>
       <c r="I39" s="7" t="n"/>
       <c r="J39" s="6" t="n"/>
     </row>
@@ -2066,31 +2074,35 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Ian V Rywalt</t>
+          <t>Suszie Campbell</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Program Manager</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>O: (407) 215-5917; M: (689) 213-9770</t>
+          <t>(951) 291-9115</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Ian.Rywalt@spectrum.com</t>
+          <t>bhavana.rao@accessonline.io</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>65 S Keller Rd, Orlando, FL 32810</t>
+          <t>9300 Arrowpoint Blvd, Charlotte, NC 28273</t>
         </is>
       </c>
       <c r="I40" s="7" t="n"/>
-      <c r="J40" s="6" t="n"/>
+      <c r="J40" s="6" t="inlineStr">
+        <is>
+          <t>Email matches Access Online's Bhavana Rao — likely a paste error, verify Suszie's real address</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2110,7 +2122,7 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Suszie Campbell</t>
+          <t>Charlamar Stephney</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2120,25 +2132,21 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>(951) 291-9115</t>
+          <t>(212) 379-5125</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>bhavana.rao@accessonline.io</t>
+          <t>Charlamar.Stephney@charter.com</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>9300 Arrowpoint Blvd, Charlotte, NC 28273</t>
+          <t>65 S Keller Rd, Orlando, FL 32810</t>
         </is>
       </c>
       <c r="I41" s="7" t="n"/>
-      <c r="J41" s="6" t="inlineStr">
-        <is>
-          <t>Email matches Access Online's Bhavana Rao — likely a paste error, verify Suszie's real address</t>
-        </is>
-      </c>
+      <c r="J41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -2158,27 +2166,27 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Charlamar Stephney</t>
+          <t>Rob Schutte</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Sr. Director</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>(212) 379-5125</t>
+          <t>(513) 386-5386</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Charlamar.Stephney@charter.com</t>
+          <t>Robert.Schutte@charter.com</t>
         </is>
       </c>
       <c r="H42" s="6" t="inlineStr">
         <is>
-          <t>65 S Keller Rd, Orlando, FL 32810</t>
+          <t>66 S Keller Rd, Orlando, FL 32810</t>
         </is>
       </c>
       <c r="I42" s="7" t="n"/>
@@ -2202,31 +2210,35 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Rob Schutte</t>
+          <t>Craig Plue</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Sr. Director</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>(513) 386-5386</t>
+          <t>(484) 629-9542</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Robert.Schutte@charter.com</t>
+          <t>craig.plue@spectrum.com</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>66 S Keller Rd, Orlando, FL 32810</t>
+          <t>67 S Keller Rd, Orlando, FL 32810</t>
         </is>
       </c>
       <c r="I43" s="7" t="n"/>
-      <c r="J43" s="6" t="n"/>
+      <c r="J43" s="6" t="inlineStr">
+        <is>
+          <t>Street numbers across this Spectrum block (65/65/66/67 S Keller Rd) look like an autofill artifact — verify each one</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2236,43 +2248,19 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Spectrum Business</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="inlineStr">
-        <is>
-          <t>Internet / Fiber</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>Craig Plue</t>
-        </is>
-      </c>
-      <c r="E44" s="5" t="inlineStr">
-        <is>
-          <t>Vice President</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>(484) 629-9542</t>
-        </is>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>craig.plue@spectrum.com</t>
-        </is>
-      </c>
-      <c r="H44" s="6" t="inlineStr">
-        <is>
-          <t>67 S Keller Rd, Orlando, FL 32810</t>
-        </is>
-      </c>
+          <t>AMI</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
+      <c r="F44" s="5" t="n"/>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="6" t="n"/>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>Street numbers across this Spectrum block (65/65/66/67 S Keller Rd) look like an autofill artifact — verify each one</t>
+          <t>From notes at bottom of old list — needs full contact info</t>
         </is>
       </c>
     </row>
@@ -2284,21 +2272,29 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>AMI</t>
+          <t>APM Services LLC</t>
         </is>
       </c>
       <c r="C45" s="6" t="n"/>
-      <c r="D45" s="5" t="n"/>
-      <c r="E45" s="5" t="n"/>
-      <c r="F45" s="5" t="n"/>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Ramón Aguirre</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>President</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>(305) 988-2350; (512) 887-7980</t>
+        </is>
+      </c>
       <c r="G45" s="6" t="n"/>
       <c r="H45" s="6" t="n"/>
       <c r="I45" s="7" t="n"/>
-      <c r="J45" s="6" t="inlineStr">
-        <is>
-          <t>From notes at bottom of old list — needs full contact info</t>
-        </is>
-      </c>
+      <c r="J45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -2314,20 +2310,20 @@
       <c r="C46" s="6" t="n"/>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Ramón Aguirre</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>President</t>
-        </is>
-      </c>
+          <t>Jacob Murphy</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="n"/>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>(305) 988-2350; (512) 887-7980</t>
-        </is>
-      </c>
-      <c r="G46" s="6" t="n"/>
+          <t>(830) 752-2023</t>
+        </is>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>murphyisme@live.com</t>
+        </is>
+      </c>
       <c r="H46" s="6" t="n"/>
       <c r="I46" s="7" t="n"/>
       <c r="J46" s="6" t="n"/>
@@ -2335,32 +2331,44 @@
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
+          <t>Supplier</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>APM Services LLC</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="n"/>
+          <t>Rapid Hotel Supplies</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>Appliances</t>
+        </is>
+      </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Jacob Murphy</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n"/>
+          <t>Andy Kumar</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>(830) 752-2023</t>
+          <t>(213) 214-1739; Office: (866) 663-3301</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>murphyisme@live.com</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="n"/>
+          <t>sales01@rapidhotelsupplies.com</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>8910 Lawndale St. Suite C, Houston, TX 77012</t>
+        </is>
+      </c>
       <c r="I47" s="7" t="n"/>
       <c r="J47" s="6" t="n"/>
     </row>
@@ -2372,37 +2380,37 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Rapid Hotel Supplies</t>
+          <t>RK Design Hospitality</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Appliances</t>
+          <t>FF&amp;E</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Andy Kumar</t>
+          <t>Ana Najera</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>(213) 214-1739; Office: (866) 663-3301</t>
+          <t>(614) 933-0300 x1006</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>sales01@rapidhotelsupplies.com</t>
+          <t>ana@rkhdesign.com</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>8910 Lawndale St. Suite C, Houston, TX 77012</t>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I48" s="7" t="n"/>
@@ -2426,22 +2434,22 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Ana Najera</t>
+          <t>Nadia Hayek</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Director of Design</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>(614) 933-0300 x1006</t>
+          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>ana@rkhdesign.com</t>
+          <t>nadia@rkhdesign.com</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
@@ -2470,31 +2478,27 @@
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Nadia Hayek</t>
-        </is>
-      </c>
-      <c r="E50" s="5" t="inlineStr">
-        <is>
-          <t>Director of Design</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
-        <is>
-          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
-        </is>
-      </c>
+          <t>Naveen Bhadari</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="n"/>
+      <c r="F50" s="5" t="n"/>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>nadia@rkhdesign.com</t>
+          <t>naveen@rkhdesign.com</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>6256 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I50" s="7" t="n"/>
-      <c r="J50" s="6" t="n"/>
+      <c r="J50" s="6" t="inlineStr">
+        <is>
+          <t>Address differs by 1 from Ana/Nadia's (6255) — verify correct suite number</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2514,25 +2518,25 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Naveen Bhadari</t>
+          <t>CB Bhandari</t>
         </is>
       </c>
       <c r="E51" s="5" t="n"/>
       <c r="F51" s="5" t="n"/>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>naveen@rkhdesign.com</t>
+          <t>cb@rkhdesign.com</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>6256 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>6257 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I51" s="7" t="n"/>
       <c r="J51" s="6" t="inlineStr">
         <is>
-          <t>Address differs by 1 from Ana/Nadia's (6255) — verify correct suite number</t>
+          <t>Address differs from Ana/Nadia's (6255) — verify correct suite number</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2548,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
+          <t>National Wholesale Hospitality</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -2554,27 +2558,27 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>CB Bhandari</t>
+          <t>Royal West</t>
         </is>
       </c>
       <c r="E52" s="5" t="n"/>
-      <c r="F52" s="5" t="n"/>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>(817) 723-5004</t>
+        </is>
+      </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>cb@rkhdesign.com</t>
+          <t>r.west@nws-inc.com</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>6257 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
         </is>
       </c>
       <c r="I52" s="7" t="n"/>
-      <c r="J52" s="6" t="inlineStr">
-        <is>
-          <t>Address differs from Ana/Nadia's (6255) — verify correct suite number</t>
-        </is>
-      </c>
+      <c r="J52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
@@ -2584,89 +2588,49 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
-          <t>National Wholesale Hospitality</t>
+          <t>Vingcard | ASSA ABLOY</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>FF&amp;E</t>
+          <t>Door locks / access</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Royal West</t>
+          <t>Leah Johnson</t>
         </is>
       </c>
       <c r="E53" s="5" t="n"/>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>(817) 723-5004</t>
+          <t>Mobile: (469) 507-0672; Tech Support: (800) 225-8464</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>r.west@nws-inc.com</t>
+          <t>leah.johnson@assaabloy.com</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+          <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
         </is>
       </c>
       <c r="I53" s="7" t="n"/>
-      <c r="J53" s="6" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Supplier</t>
-        </is>
-      </c>
-      <c r="B54" s="5" t="inlineStr">
-        <is>
-          <t>Vingcard | ASSA ABLOY</t>
-        </is>
-      </c>
-      <c r="C54" s="6" t="inlineStr">
-        <is>
-          <t>Door locks / access</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>Leah Johnson</t>
-        </is>
-      </c>
-      <c r="E54" s="5" t="n"/>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>Mobile: (469) 507-0672; Tech Support: (800) 225-8464</t>
-        </is>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
-        <is>
-          <t>leah.johnson@assaabloy.com</t>
-        </is>
-      </c>
-      <c r="H54" s="6" t="inlineStr">
-        <is>
-          <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
-        </is>
-      </c>
-      <c r="I54" s="7" t="n"/>
-      <c r="J54" s="6" t="inlineStr">
+      <c r="J53" s="6" t="inlineStr">
         <is>
           <t>From notes at bottom of old list — assaabloyglobalsolutions.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:H54">
+  <conditionalFormatting sqref="B6:H53">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:H54">
+  <conditionalFormatting sqref="C6:H53">
     <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(C6),$B6&lt;&gt;"")</formula>
     </cfRule>

</xml_diff>

<commit_message>
Add owner/developer and Hilton brand contacts
Adds four contacts:
- Ken Patel, Project Manager, JD Design and Developers LLC
- Kamlesh Patel and Vipal Patel, owners, Vibrant Services LLC
- Justine Chiang, Senior Manager North America ADC, Hilton All Suites Brands

Adds a 'Brand / Franchisor' option to the Category dropdown so the Hilton
brand contact is not miscategorized under an existing trade role.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -201,8 +201,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J53" headerRowCount="1">
-  <autoFilter ref="A5:J53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ContactsTable" displayName="ContactsTable" ref="A5:J57" headerRowCount="1">
+  <autoFilter ref="A5:J57"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Category"/>
     <tableColumn id="2" name="Organization"/>
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -599,236 +599,216 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Engineer</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="n"/>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>JD Design and Developers LLC</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Development / project management</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ken Patel</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>(903) 705-3336</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>pm.jddevelopers@gmail.com</t>
+        </is>
+      </c>
       <c r="H6" s="6" t="n"/>
       <c r="I6" s="7" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Open slot — add current engineer of record</t>
-        </is>
-      </c>
+      <c r="J6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Architect</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>MWT</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Architecture</t>
-        </is>
-      </c>
+          <t>Vibrant Services, LLC</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Anita Bansal</t>
+          <t>Kamlesh Patel</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>AIA, NCARB</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>(716) 435-0019</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>anita@mwtusa.com</t>
-        </is>
-      </c>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="6" t="n"/>
       <c r="H7" s="6" t="n"/>
       <c r="I7" s="7" t="n"/>
-      <c r="J7" s="6" t="n"/>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>Confirm role on this project; fill in phone and email</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Triun, LLC</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>General contractor</t>
-        </is>
-      </c>
+          <t>Vibrant Services, LLC</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Edward R. De La Garza</t>
+          <t>Vipal Patel</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>(210) 572-4900</t>
+          <t>(575) 937-1954</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>edelagarza@triunco.com</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
-        </is>
-      </c>
+          <t>vipal.m.patel@gmail.com</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
       <c r="I8" s="7" t="n"/>
-      <c r="J8" s="6" t="n"/>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Confirm role on this project</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
+          <t>Brand / Franchisor</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Triun, LLC</t>
+          <t>Hilton</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>General contractor</t>
+          <t>Brand standards / ADC review</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Cesar Esquivel</t>
+          <t>Justine Chiang</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>General Superintendent</t>
+          <t>Senior Manager – North America, Architecture Design &amp; Construction, All Suites Brands</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>(210) 718-1001</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>cesquivel@triunco.com</t>
-        </is>
-      </c>
+          <t>(512) 434-9028</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
+          <t>Austin, TX</t>
         </is>
       </c>
       <c r="I9" s="7" t="n"/>
-      <c r="J9" s="6" t="n"/>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>No email provided — get direct address; hilton.com</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Triun, LLC</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>General contractor</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Joaquin Gomez</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Superintendent</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>(830) 335-0522</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>jgomez@triunco.com</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
-        </is>
-      </c>
+          <t>Engineer</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
       <c r="I10" s="7" t="n"/>
-      <c r="J10" s="6" t="n"/>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>Open slot — add current engineer of record</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Contractor (GC)</t>
+          <t>Architect</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Triun, LLC</t>
+          <t>MWT</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>General contractor</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Morgan Davis</t>
+          <t>Anita Bansal</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Project Manager I</t>
+          <t>AIA, NCARB</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>(512) 771-2329</t>
+          <t>(716) 435-0019</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>mdavis@triunco.com</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
-        </is>
-      </c>
+          <t>anita@mwtusa.com</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="n"/>
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="6" t="n"/>
     </row>
@@ -850,22 +830,22 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Austin Jones</t>
+          <t>Edward R. De La Garza</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Assistant Project Manager</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>(210) 834-9687</t>
+          <t>(210) 572-4900</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>ajones@triunco.com</t>
+          <t>edelagarza@triunco.com</t>
         </is>
       </c>
       <c r="H12" s="6" t="inlineStr">
@@ -879,42 +859,42 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Contractor (GC)</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Iceberg Heating &amp; Air Conditioning</t>
+          <t>Triun, LLC</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Mechanical / HVAC</t>
+          <t>General contractor</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Jorge Garcia</t>
+          <t>Cesar Esquivel</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>General Superintendent</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>(817) 920-9950</t>
+          <t>(210) 718-1001</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
+          <t>cesquivel@triunco.com</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
+          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
         </is>
       </c>
       <c r="I13" s="7" t="n"/>
@@ -923,42 +903,42 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Contractor (GC)</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Iceberg Heating &amp; Air Conditioning</t>
+          <t>Triun, LLC</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Mechanical / HVAC</t>
+          <t>General contractor</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Andrea Garcia</t>
+          <t>Joaquin Gomez</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>Estimator</t>
+          <t>Superintendent</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>(817) 920-9950</t>
+          <t>(830) 335-0522</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>estimating@icebergair.com</t>
+          <t>jgomez@triunco.com</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>1220 Oak Knoll Dr. Suite 200, Fort Worth, TX 76117</t>
+          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
         </is>
       </c>
       <c r="I14" s="7" t="n"/>
@@ -967,42 +947,42 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Contractor (GC)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>United Electric</t>
+          <t>Triun, LLC</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>General contractor</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Manuel Hernandez</t>
+          <t>Morgan Davis</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Project Manager I</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>(956) 309-4209</t>
+          <t>(512) 771-2329</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>manuel@unitedelectricrgv.com</t>
+          <t>mdavis@triunco.com</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>4624 Martinal Road, Brownsville, TX 78526</t>
+          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
         </is>
       </c>
       <c r="I15" s="7" t="n"/>
@@ -1011,42 +991,42 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>MEP</t>
+          <t>Contractor (GC)</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
+          <t>Triun, LLC</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>General contractor</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Larry Sanchez</t>
+          <t>Austin Jones</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Assistant Project Manager</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>(830) 513-1789</t>
+          <t>(210) 834-9687</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>larrysplumbing@live.com</t>
+          <t>ajones@triunco.com</t>
         </is>
       </c>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
+          <t>4242 Medical Dr., Suite 1200, San Antonio, TX 78229</t>
         </is>
       </c>
       <c r="I16" s="7" t="n"/>
@@ -1060,85 +1040,81 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
+          <t>Iceberg Heating &amp; Air Conditioning</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Mechanical / HVAC</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Jay Hernandaz</t>
+          <t>Jorge Garcia</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>Foreman</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>(830) 513-1789</t>
+          <t>(817) 920-9950</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>larrysplumbing@live.com</t>
+          <t>jorgejr@icebergair.com; estimating@icebergair.com</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
+          <t>4001 McCart Ave., Fort Worth, TX 76110</t>
         </is>
       </c>
       <c r="I17" s="7" t="n"/>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>From notes at bottom of old list — verify name spelling and get direct number</t>
-        </is>
-      </c>
+      <c r="J17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Steel Tech USA</t>
+          <t>Iceberg Heating &amp; Air Conditioning</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Steel erection</t>
+          <t>Mechanical / HVAC</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Yalcin Kucukkomurler</t>
+          <t>Andrea Garcia</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>Director of Engineering</t>
+          <t>Estimator</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>(561) 906-2840</t>
+          <t>(817) 920-9950</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>yalcin@steeltechusa.com</t>
+          <t>estimating@icebergair.com</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
+          <t>1220 Oak Knoll Dr. Suite 200, Fort Worth, TX 76117</t>
         </is>
       </c>
       <c r="I18" s="7" t="n"/>
@@ -1147,42 +1123,42 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>A/E Hiller &amp; Sons Inc.</t>
+          <t>United Electric</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Concrete; parking lot striping &amp; signage; ADA pavers</t>
+          <t>Electrical</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>Christopher Hiller</t>
+          <t>Manuel Hernandez</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>(830) 773-9156</t>
+          <t>(956) 309-4209</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>cw_hiller@yahoo.com</t>
+          <t>manuel@unitedelectricrgv.com</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>P.O. Box 557, Eagle Pass, TX 78852</t>
+          <t>4624 Martinal Road, Brownsville, TX 78526</t>
         </is>
       </c>
       <c r="I19" s="7" t="n"/>
@@ -1191,18 +1167,22 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>JC Enterprises</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="n"/>
+          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Isaac Chapa</t>
+          <t>Larry Sanchez</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1212,17 +1192,17 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>(830) 968-1857</t>
+          <t>(830) 513-1789</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>jcenterprises@yahoo.com</t>
+          <t>larrysplumbing@live.com</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>2254 Foothills St., Eagle Pass, TX 78852</t>
+          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I20" s="7" t="n"/>
@@ -1231,86 +1211,90 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
+          <t>MEP</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Texas Fire Services, LLC</t>
+          <t>Larry's Commercial &amp; Residential Plumbing, LLC</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Fire protection</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Rodney Jackson</t>
+          <t>Jay Hernandaz</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Foreman</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>(830) 609-9090</t>
+          <t>(830) 513-1789</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>rod@texasfireservices.net</t>
+          <t>larrysplumbing@live.com</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>1260 FM 1863, Building 2, New Braunfels, TX 78132</t>
+          <t>2615 El Indio Hwy., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I21" s="7" t="n"/>
-      <c r="J21" s="6" t="n"/>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>From notes at bottom of old list — verify name spelling and get direct number</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Subcontractor</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>TK Elevator Corporation</t>
+          <t>Steel Tech USA</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Elevator</t>
+          <t>Steel erection</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>WH (Joey) Hawkins Jr.</t>
+          <t>Yalcin Kucukkomurler</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Director of Engineering</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>(210) 669-4818</t>
+          <t>(561) 906-2840</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>joey.hawkins@tkelevator.com</t>
+          <t>yalcin@steeltechusa.com</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>3660 Thousand Oaks, Suite 210, San Antonio, TX 78247</t>
+          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
         </is>
       </c>
       <c r="I22" s="7" t="n"/>
@@ -1324,37 +1308,37 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Irontek Metal Works</t>
+          <t>A/E Hiller &amp; Sons Inc.</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Misc. metals</t>
+          <t>Concrete; parking lot striping &amp; signage; ADA pavers</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Johnny Pina</t>
+          <t>Christopher Hiller</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>President</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>(512) 633-5140</t>
+          <t>(830) 773-9156</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>irontekmetalworks@gmail.com</t>
+          <t>cw_hiller@yahoo.com</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>213 Goldenrod, San Marcos, TX 78666</t>
+          <t>P.O. Box 557, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I23" s="7" t="n"/>
@@ -1368,17 +1352,13 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>The Montecito</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Stucco / plastering</t>
-        </is>
-      </c>
+          <t>JC Enterprises</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="n"/>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Victor A. Rodriguez</t>
+          <t>Isaac Chapa</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1388,17 +1368,17 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>(940) 600-8106</t>
+          <t>(830) 968-1857</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>plasteringstuccoirdallas@gmail.com</t>
+          <t>jcenterprises@yahoo.com</t>
         </is>
       </c>
       <c r="H24" s="6" t="inlineStr">
         <is>
-          <t>5517 Rio Rd., Denton, TX 76208</t>
+          <t>2254 Foothills St., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I24" s="7" t="n"/>
@@ -1412,17 +1392,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Keen Glass Solutions</t>
+          <t>Texas Fire Services, LLC</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Glass &amp; glazing</t>
+          <t>Fire protection</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Joe Wilkinson</t>
+          <t>Rodney Jackson</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1432,17 +1412,17 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>(214) 673-1761</t>
+          <t>(830) 609-9090</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>sales@keen-glass.org</t>
+          <t>rod@texasfireservices.net</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>3923 Morse St. #116, Denton, TX 76208</t>
+          <t>1260 FM 1863, Building 2, New Braunfels, TX 78132</t>
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
@@ -1456,17 +1436,17 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Thermal Guard Roofing</t>
+          <t>TK Elevator Corporation</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>TPO roofing</t>
+          <t>Elevator</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Quinton Rockwell</t>
+          <t>WH (Joey) Hawkins Jr.</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1476,17 +1456,17 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>(817) 909-9884</t>
+          <t>(210) 669-4818</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>quinton@thermalguardroofing.com</t>
+          <t>joey.hawkins@tkelevator.com</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>P.O. Box 1026, Argyle, TX 76226</t>
+          <t>3660 Thousand Oaks, Suite 210, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I26" s="7" t="n"/>
@@ -1500,17 +1480,17 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Security Integrated</t>
+          <t>Irontek Metal Works</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Security systems</t>
+          <t>Misc. metals</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Randy Jasik</t>
+          <t>Johnny Pina</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1520,17 +1500,17 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>(210) 519-5009</t>
+          <t>(512) 633-5140</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>team@siinc.systems</t>
+          <t>irontekmetalworks@gmail.com</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>14080 Nacogdoches Rd. #536, San Antonio, TX 78247</t>
+          <t>213 Goldenrod, San Marcos, TX 78666</t>
         </is>
       </c>
       <c r="I27" s="7" t="n"/>
@@ -1544,17 +1524,17 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Tormax USA, LLC</t>
+          <t>The Montecito</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Automatic glass doors</t>
+          <t>Stucco / plastering</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Chris Valadez</t>
+          <t>Victor A. Rodriguez</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1564,17 +1544,17 @@
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>(210) 362-4887</t>
+          <t>(940) 600-8106</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>cvaladez@tormaxusa.com</t>
+          <t>plasteringstuccoirdallas@gmail.com</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>12859 Wetmore Road, San Antonio, TX 78247</t>
+          <t>5517 Rio Rd., Denton, TX 76208</t>
         </is>
       </c>
       <c r="I28" s="7" t="n"/>
@@ -1588,17 +1568,17 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Steel Tech USA</t>
+          <t>Keen Glass Solutions</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Steel fabrication</t>
+          <t>Glass &amp; glazing</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Edward Tekin</t>
+          <t>Joe Wilkinson</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1608,17 +1588,17 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>(254) 368-7956</t>
+          <t>(214) 673-1761</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>edward@steeltechusa.com</t>
+          <t>sales@keen-glass.org</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
+          <t>3923 Morse St. #116, Denton, TX 76208</t>
         </is>
       </c>
       <c r="I29" s="7" t="n"/>
@@ -1632,17 +1612,17 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Texas Chutes</t>
+          <t>Thermal Guard Roofing</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Trash / linen chutes</t>
+          <t>TPO roofing</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Gerry Whitaker</t>
+          <t>Quinton Rockwell</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1652,17 +1632,17 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>(830) 964-3102</t>
+          <t>(817) 909-9884</t>
         </is>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>gerry@texaschutes.com</t>
+          <t>quinton@thermalguardroofing.com</t>
         </is>
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>14812 South Access Rd. #A, Canyon Lake, TX 78133</t>
+          <t>P.O. Box 1026, Argyle, TX 76226</t>
         </is>
       </c>
       <c r="I30" s="7" t="n"/>
@@ -1676,41 +1656,41 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Texas Chutes</t>
+          <t>Security Integrated</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Trash / linen chutes</t>
+          <t>Security systems</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Annalisa Call</t>
+          <t>Randy Jasik</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Administrative Assistant</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>(830) 964-3102</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="n"/>
+          <t>(210) 519-5009</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>team@siinc.systems</t>
+        </is>
+      </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>14812 S. Access Road, Unit A, Canyon Lake, TX 78133</t>
+          <t>14080 Nacogdoches Rd. #536, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I31" s="7" t="n"/>
-      <c r="J31" s="6" t="inlineStr">
-        <is>
-          <t>www.texaschutes.com</t>
-        </is>
-      </c>
+      <c r="J31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -1720,17 +1700,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Keepers Construction</t>
+          <t>Tormax USA, LLC</t>
         </is>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Flooring</t>
+          <t>Automatic glass doors</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Justin Allen Perez</t>
+          <t>Chris Valadez</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1740,17 +1720,17 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>(210) 909-3250</t>
+          <t>(210) 362-4887</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>keeperconst@gmail.com</t>
+          <t>cvaladez@tormaxusa.com</t>
         </is>
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
+          <t>12859 Wetmore Road, San Antonio, TX 78247</t>
         </is>
       </c>
       <c r="I32" s="7" t="n"/>
@@ -1764,17 +1744,17 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>Velasquez Pool</t>
+          <t>Steel Tech USA</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Pool</t>
+          <t>Steel fabrication</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Sabino Velasquez</t>
+          <t>Edward Tekin</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1784,17 +1764,17 @@
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>(830) 352-4026</t>
+          <t>(254) 368-7956</t>
         </is>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>velasquezpools@yahoo.com</t>
+          <t>edward@steeltechusa.com</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
+          <t>500 Huffines Blvd., Lewisville, TX 75056</t>
         </is>
       </c>
       <c r="I33" s="7" t="n"/>
@@ -1808,17 +1788,17 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Cemplex Group</t>
+          <t>Texas Chutes</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Gypsum floor underlayment</t>
+          <t>Trash / linen chutes</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Shane Kuempel</t>
+          <t>Gerry Whitaker</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1828,17 +1808,17 @@
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>(817) 760-9457</t>
+          <t>(830) 964-3102</t>
         </is>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>skuempel@cemplexgroup.com</t>
+          <t>gerry@texaschutes.com</t>
         </is>
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
+          <t>14812 South Access Rd. #A, Canyon Lake, TX 78133</t>
         </is>
       </c>
       <c r="I34" s="7" t="n"/>
@@ -1852,37 +1832,41 @@
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Access Online Inc</t>
+          <t>Texas Chutes</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Data / low voltage</t>
+          <t>Trash / linen chutes</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Rameez</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="n"/>
+          <t>Annalisa Call</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Administrative Assistant</t>
+        </is>
+      </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>(847) 306-3777 Ext. 8205</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>rameez@accessonline.io</t>
-        </is>
-      </c>
+          <t>(830) 964-3102</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="n"/>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>2130 Foster Ave., Wheeling, IL 60090</t>
+          <t>14812 S. Access Road, Unit A, Canyon Lake, TX 78133</t>
         </is>
       </c>
       <c r="I35" s="7" t="n"/>
-      <c r="J35" s="6" t="n"/>
+      <c r="J35" s="6" t="inlineStr">
+        <is>
+          <t>www.texaschutes.com</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -1892,37 +1876,37 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>Access Online Inc</t>
+          <t>Keepers Construction</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Data / low voltage</t>
+          <t>Flooring</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Bhavana Rao</t>
+          <t>Justin Allen Perez</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Project Coordinator</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Direct: (847) 881-3681; Office: (847) 306-3777 Ext. 8603</t>
+          <t>(210) 909-3250</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>bhavana.rao@accessonline.io</t>
+          <t>keeperconst@gmail.com</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>2130 Foster Ave., Wheeling, IL 60090</t>
+          <t>2016 E Garrison St., Ste 24, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I36" s="7" t="n"/>
@@ -1936,17 +1920,17 @@
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>The Green Company</t>
+          <t>Velasquez Pool</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Landscaping</t>
+          <t>Pool</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Jorge Cavazos</t>
+          <t>Sabino Velasquez</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1956,17 +1940,17 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>(830) 335-2488</t>
+          <t>(830) 352-4026</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>management@thegreencoep.com</t>
+          <t>velasquezpools@yahoo.com</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>126 Concho Street, Eagle Pass, TX 78852</t>
+          <t>1586 Valerie Dr., Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I37" s="7" t="n"/>
@@ -1980,35 +1964,39 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Pinnacle Communications</t>
+          <t>Cemplex Group</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Communications</t>
+          <t>Gypsum floor underlayment</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Trista Stillwagon</t>
+          <t>Shane Kuempel</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Project Coordinator</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
+          <t>(817) 760-9457</t>
         </is>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>tstillwagon@pinn360.com</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="n"/>
+          <t>skuempel@cemplexgroup.com</t>
+        </is>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
+        <is>
+          <t>2135 Wald Rd., New Braunfels, TX 78132</t>
+        </is>
+      </c>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="6" t="n"/>
     </row>
@@ -2020,37 +2008,33 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Spectrum Business</t>
+          <t>Access Online Inc</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Internet / Fiber</t>
+          <t>Data / low voltage</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Ian V Rywalt</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Program Manager</t>
-        </is>
-      </c>
+          <t>Rameez</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="n"/>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>O: (407) 215-5917; M: (689) 213-9770</t>
+          <t>(847) 306-3777 Ext. 8205</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Ian.Rywalt@spectrum.com</t>
+          <t>rameez@accessonline.io</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>65 S Keller Rd, Orlando, FL 32810</t>
+          <t>2130 Foster Ave., Wheeling, IL 60090</t>
         </is>
       </c>
       <c r="I39" s="7" t="n"/>
@@ -2064,27 +2048,27 @@
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Spectrum Business</t>
+          <t>Access Online Inc</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Internet / Fiber</t>
+          <t>Data / low voltage</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Suszie Campbell</t>
+          <t>Bhavana Rao</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Project Coordinator</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>(951) 291-9115</t>
+          <t>Direct: (847) 881-3681; Office: (847) 306-3777 Ext. 8603</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
@@ -2094,15 +2078,11 @@
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>9300 Arrowpoint Blvd, Charlotte, NC 28273</t>
+          <t>2130 Foster Ave., Wheeling, IL 60090</t>
         </is>
       </c>
       <c r="I40" s="7" t="n"/>
-      <c r="J40" s="6" t="inlineStr">
-        <is>
-          <t>Email matches Access Online's Bhavana Rao — likely a paste error, verify Suszie's real address</t>
-        </is>
-      </c>
+      <c r="J40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
@@ -2112,37 +2092,37 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Spectrum Business</t>
+          <t>The Green Company</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Internet / Fiber</t>
+          <t>Landscaping</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Charlamar Stephney</t>
+          <t>Jorge Cavazos</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>(212) 379-5125</t>
+          <t>(830) 335-2488</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Charlamar.Stephney@charter.com</t>
+          <t>management@thegreencoep.com</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>65 S Keller Rd, Orlando, FL 32810</t>
+          <t>126 Concho Street, Eagle Pass, TX 78852</t>
         </is>
       </c>
       <c r="I41" s="7" t="n"/>
@@ -2156,39 +2136,35 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Spectrum Business</t>
+          <t>Pinnacle Communications</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Internet / Fiber</t>
+          <t>Communications</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Rob Schutte</t>
+          <t>Trista Stillwagon</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Sr. Director</t>
+          <t>Project Coordinator</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>(513) 386-5386</t>
+          <t>Main: (800) 644-9101; Direct: (240) 912-2546</t>
         </is>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>Robert.Schutte@charter.com</t>
-        </is>
-      </c>
-      <c r="H42" s="6" t="inlineStr">
-        <is>
-          <t>66 S Keller Rd, Orlando, FL 32810</t>
-        </is>
-      </c>
+          <t>tstillwagon@pinn360.com</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="n"/>
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="6" t="n"/>
     </row>
@@ -2210,35 +2186,31 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Craig Plue</t>
+          <t>Ian V Rywalt</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Vice President</t>
+          <t>Program Manager</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>(484) 629-9542</t>
+          <t>O: (407) 215-5917; M: (689) 213-9770</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>craig.plue@spectrum.com</t>
+          <t>Ian.Rywalt@spectrum.com</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>67 S Keller Rd, Orlando, FL 32810</t>
+          <t>65 S Keller Rd, Orlando, FL 32810</t>
         </is>
       </c>
       <c r="I43" s="7" t="n"/>
-      <c r="J43" s="6" t="inlineStr">
-        <is>
-          <t>Street numbers across this Spectrum block (65/65/66/67 S Keller Rd) look like an autofill artifact — verify each one</t>
-        </is>
-      </c>
+      <c r="J43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -2248,19 +2220,43 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>AMI</t>
-        </is>
-      </c>
-      <c r="C44" s="6" t="n"/>
-      <c r="D44" s="5" t="n"/>
-      <c r="E44" s="5" t="n"/>
-      <c r="F44" s="5" t="n"/>
-      <c r="G44" s="6" t="n"/>
-      <c r="H44" s="6" t="n"/>
+          <t>Spectrum Business</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Internet / Fiber</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Suszie Campbell</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>(951) 291-9115</t>
+        </is>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>bhavana.rao@accessonline.io</t>
+        </is>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
+        <is>
+          <t>9300 Arrowpoint Blvd, Charlotte, NC 28273</t>
+        </is>
+      </c>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="6" t="inlineStr">
         <is>
-          <t>From notes at bottom of old list — needs full contact info</t>
+          <t>Email matches Access Online's Bhavana Rao — likely a paste error, verify Suszie's real address</t>
         </is>
       </c>
     </row>
@@ -2272,27 +2268,39 @@
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>APM Services LLC</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="n"/>
+          <t>Spectrum Business</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Internet / Fiber</t>
+        </is>
+      </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Ramón Aguirre</t>
+          <t>Charlamar Stephney</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>President</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>(305) 988-2350; (512) 887-7980</t>
-        </is>
-      </c>
-      <c r="G45" s="6" t="n"/>
-      <c r="H45" s="6" t="n"/>
+          <t>(212) 379-5125</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Charlamar.Stephney@charter.com</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>65 S Keller Rd, Orlando, FL 32810</t>
+        </is>
+      </c>
       <c r="I45" s="7" t="n"/>
       <c r="J45" s="6" t="n"/>
     </row>
@@ -2304,201 +2312,177 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>APM Services LLC</t>
-        </is>
-      </c>
-      <c r="C46" s="6" t="n"/>
+          <t>Spectrum Business</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>Internet / Fiber</t>
+        </is>
+      </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Jacob Murphy</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="n"/>
+          <t>Rob Schutte</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Sr. Director</t>
+        </is>
+      </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>(830) 752-2023</t>
+          <t>(513) 386-5386</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>murphyisme@live.com</t>
-        </is>
-      </c>
-      <c r="H46" s="6" t="n"/>
+          <t>Robert.Schutte@charter.com</t>
+        </is>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
+        <is>
+          <t>66 S Keller Rd, Orlando, FL 32810</t>
+        </is>
+      </c>
       <c r="I46" s="7" t="n"/>
       <c r="J46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Subcontractor</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>Rapid Hotel Supplies</t>
+          <t>Spectrum Business</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Appliances</t>
+          <t>Internet / Fiber</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Andy Kumar</t>
+          <t>Craig Plue</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>Vice President</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>(213) 214-1739; Office: (866) 663-3301</t>
+          <t>(484) 629-9542</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>sales01@rapidhotelsupplies.com</t>
+          <t>craig.plue@spectrum.com</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>8910 Lawndale St. Suite C, Houston, TX 77012</t>
+          <t>67 S Keller Rd, Orlando, FL 32810</t>
         </is>
       </c>
       <c r="I47" s="7" t="n"/>
-      <c r="J47" s="6" t="n"/>
+      <c r="J47" s="6" t="inlineStr">
+        <is>
+          <t>Street numbers across this Spectrum block (65/65/66/67 S Keller Rd) look like an autofill artifact — verify each one</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Subcontractor</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
-        </is>
-      </c>
-      <c r="C48" s="6" t="inlineStr">
-        <is>
-          <t>FF&amp;E</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>Ana Najera</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="inlineStr">
-        <is>
-          <t>Project Manager</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>(614) 933-0300 x1006</t>
-        </is>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>ana@rkhdesign.com</t>
-        </is>
-      </c>
-      <c r="H48" s="6" t="inlineStr">
-        <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
-        </is>
-      </c>
+          <t>AMI</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
+      <c r="F48" s="5" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="6" t="n"/>
       <c r="I48" s="7" t="n"/>
-      <c r="J48" s="6" t="n"/>
+      <c r="J48" s="6" t="inlineStr">
+        <is>
+          <t>From notes at bottom of old list — needs full contact info</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Subcontractor</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
-        </is>
-      </c>
-      <c r="C49" s="6" t="inlineStr">
-        <is>
-          <t>FF&amp;E</t>
-        </is>
-      </c>
+          <t>APM Services LLC</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="n"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Nadia Hayek</t>
+          <t>Ramón Aguirre</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Director of Design</t>
+          <t>President</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
-        </is>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>nadia@rkhdesign.com</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
-        <is>
-          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
-        </is>
-      </c>
+          <t>(305) 988-2350; (512) 887-7980</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="6" t="n"/>
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Supplier</t>
+          <t>Subcontractor</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>FF&amp;E</t>
-        </is>
-      </c>
+          <t>APM Services LLC</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n"/>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Naveen Bhadari</t>
+          <t>Jacob Murphy</t>
         </is>
       </c>
       <c r="E50" s="5" t="n"/>
-      <c r="F50" s="5" t="n"/>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>(830) 752-2023</t>
+        </is>
+      </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>naveen@rkhdesign.com</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>6256 Corporate Center Drive, Dublin, OH 43016</t>
-        </is>
-      </c>
+          <t>murphyisme@live.com</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="n"/>
       <c r="I50" s="7" t="n"/>
-      <c r="J50" s="6" t="inlineStr">
-        <is>
-          <t>Address differs by 1 from Ana/Nadia's (6255) — verify correct suite number</t>
-        </is>
-      </c>
+      <c r="J50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
@@ -2508,37 +2492,41 @@
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>RK Design Hospitality</t>
+          <t>Rapid Hotel Supplies</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>FF&amp;E</t>
+          <t>Appliances</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>CB Bhandari</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="n"/>
-      <c r="F51" s="5" t="n"/>
+          <t>Andy Kumar</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>(213) 214-1739; Office: (866) 663-3301</t>
+        </is>
+      </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>cb@rkhdesign.com</t>
+          <t>sales01@rapidhotelsupplies.com</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>6257 Corporate Center Drive, Dublin, OH 43016</t>
+          <t>8910 Lawndale St. Suite C, Houston, TX 77012</t>
         </is>
       </c>
       <c r="I51" s="7" t="n"/>
-      <c r="J51" s="6" t="inlineStr">
-        <is>
-          <t>Address differs from Ana/Nadia's (6255) — verify correct suite number</t>
-        </is>
-      </c>
+      <c r="J51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -2548,7 +2536,7 @@
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>National Wholesale Hospitality</t>
+          <t>RK Design Hospitality</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
@@ -2558,23 +2546,27 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Royal West</t>
-        </is>
-      </c>
-      <c r="E52" s="5" t="n"/>
+          <t>Ana Najera</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>(817) 723-5004</t>
+          <t>(614) 933-0300 x1006</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>r.west@nws-inc.com</t>
+          <t>ana@rkhdesign.com</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
         </is>
       </c>
       <c r="I52" s="7" t="n"/>
@@ -2588,56 +2580,220 @@
       </c>
       <c r="B53" s="5" t="inlineStr">
         <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Nadia Hayek</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Director of Design</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Cell: (312) 825-6146; Office: (614) 933-0300</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>nadia@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>6255 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I53" s="7" t="n"/>
+      <c r="J53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Naveen Bhadari</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="n"/>
+      <c r="F54" s="5" t="n"/>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>naveen@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>6256 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="n"/>
+      <c r="J54" s="6" t="inlineStr">
+        <is>
+          <t>Address differs by 1 from Ana/Nadia's (6255) — verify correct suite number</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>RK Design Hospitality</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>CB Bhandari</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="n"/>
+      <c r="F55" s="5" t="n"/>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>cb@rkhdesign.com</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>6257 Corporate Center Drive, Dublin, OH 43016</t>
+        </is>
+      </c>
+      <c r="I55" s="7" t="n"/>
+      <c r="J55" s="6" t="inlineStr">
+        <is>
+          <t>Address differs from Ana/Nadia's (6255) — verify correct suite number</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>National Wholesale Hospitality</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>FF&amp;E</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Royal West</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="n"/>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>(817) 723-5004</t>
+        </is>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>r.west@nws-inc.com</t>
+        </is>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
+        <is>
+          <t>4108 Keller Hicks Road, Building B, Keller, TX 76248</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="n"/>
+      <c r="J56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Supplier</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
           <t>Vingcard | ASSA ABLOY</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Door locks / access</t>
         </is>
       </c>
-      <c r="D53" s="5" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>Leah Johnson</t>
         </is>
       </c>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="E57" s="5" t="n"/>
+      <c r="F57" s="5" t="inlineStr">
         <is>
           <t>Mobile: (469) 507-0672; Tech Support: (800) 225-8464</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>leah.johnson@assaabloy.com</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>2925 E. Plano Pkwy, Plano, TX 75074</t>
         </is>
       </c>
-      <c r="I53" s="7" t="n"/>
-      <c r="J53" s="6" t="inlineStr">
+      <c r="I57" s="7" t="n"/>
+      <c r="J57" s="6" t="inlineStr">
         <is>
           <t>assaabloyglobalsolutions.com</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B6:H53">
+  <conditionalFormatting sqref="B6:H57">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(B6),$A6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:H53">
+  <conditionalFormatting sqref="C6:H57">
     <cfRule type="expression" priority="2" dxfId="0" stopIfTrue="0">
       <formula>AND(ISBLANK(C6),$B6&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="A6:A300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid category" error="Pick a category from the list." type="list">
-      <formula1>"Owner,Engineer,Architect,Contractor (GC),MEP,Structural,Subcontractor,Supplier,Consultant,Inspector / AHJ"</formula1>
+      <formula1>"Owner,Brand / Franchisor,Engineer,Architect,Contractor (GC),MEP,Structural,Subcontractor,Supplier,Consultant,Inspector / AHJ"</formula1>
     </dataValidation>
     <dataValidation sqref="I6:I300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,N/A"</formula1>

</xml_diff>

<commit_message>
Add Texas Fire Services licenses and cell to Rodney Jackson's row
Records the four Texas licenses (RME, alarm, sprinkler, security) and
AUTOCALL/CWSI distributor status in Notes, and adds the 956 cell number
flagged for confirmation since the signature block named no contact.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UdvWW191kBuYgxuQer2e2E
</commit_message>
<xml_diff>
--- a/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
+++ b/docs/H2SEP-PhII_Contact-List_2026-08-14.xlsx
@@ -1412,7 +1412,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>(830) 609-9090</t>
+          <t>(830) 609-9090; C: (956) 376-7054</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -1426,7 +1426,11 @@
         </is>
       </c>
       <c r="I25" s="7" t="n"/>
-      <c r="J25" s="6" t="n"/>
+      <c r="J25" s="6" t="inlineStr">
+        <is>
+          <t>Cell (956) 376-7054 came off the company signature block — confirm it is Rodney's. TX licenses: RME G 1768429; Alarm ACR-2368235; Sprinkler SCR-G-2398977; Security B09419101. Authorized distributor of AUTOCALL/CWSI</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">

</xml_diff>